<commit_message>
check list fixed. SUPER アカウントを追加
</commit_message>
<xml_diff>
--- a/docs/db-design_document.xlsx
+++ b/docs/db-design_document.xlsx
@@ -139,7 +139,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -168,6 +168,34 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -179,7 +207,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -263,6 +291,8 @@
     <xf numFmtId="0" fontId="14" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -555,7 +585,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Ver 2.0 — 2026-05-24 更新 | 全24テーブル</t>
         </is>
@@ -1753,12 +1783,12 @@
           <t>▶ roles</t>
         </is>
       </c>
-      <c r="B4" s="26" t="n"/>
-      <c r="C4" s="26" t="n"/>
-      <c r="D4" s="26" t="n"/>
-      <c r="E4" s="26" t="n"/>
-      <c r="F4" s="26" t="n"/>
-      <c r="G4" s="26" t="n"/>
+      <c r="B4" s="29" t="n"/>
+      <c r="C4" s="29" t="n"/>
+      <c r="D4" s="29" t="n"/>
+      <c r="E4" s="29" t="n"/>
+      <c r="F4" s="29" t="n"/>
+      <c r="G4" s="30" t="n"/>
     </row>
     <row r="5" ht="15" customHeight="1" s="12">
       <c r="A5" s="26" t="inlineStr">
@@ -1931,12 +1961,12 @@
           <t>▶ users</t>
         </is>
       </c>
-      <c r="B10" s="26" t="n"/>
-      <c r="C10" s="26" t="n"/>
-      <c r="D10" s="26" t="n"/>
-      <c r="E10" s="26" t="n"/>
-      <c r="F10" s="26" t="n"/>
-      <c r="G10" s="26" t="n"/>
+      <c r="B10" s="29" t="n"/>
+      <c r="C10" s="29" t="n"/>
+      <c r="D10" s="29" t="n"/>
+      <c r="E10" s="29" t="n"/>
+      <c r="F10" s="29" t="n"/>
+      <c r="G10" s="30" t="n"/>
     </row>
     <row r="11" ht="15" customHeight="1" s="12">
       <c r="A11" s="26" t="inlineStr">
@@ -2369,12 +2399,12 @@
           <t>▶ pets</t>
         </is>
       </c>
-      <c r="B24" s="26" t="n"/>
-      <c r="C24" s="26" t="n"/>
-      <c r="D24" s="26" t="n"/>
-      <c r="E24" s="26" t="n"/>
-      <c r="F24" s="26" t="n"/>
-      <c r="G24" s="26" t="n"/>
+      <c r="B24" s="29" t="n"/>
+      <c r="C24" s="29" t="n"/>
+      <c r="D24" s="29" t="n"/>
+      <c r="E24" s="29" t="n"/>
+      <c r="F24" s="29" t="n"/>
+      <c r="G24" s="30" t="n"/>
     </row>
     <row r="25" ht="15" customHeight="1" s="12">
       <c r="A25" s="26" t="inlineStr">
@@ -2807,12 +2837,12 @@
           <t>▶ health_records</t>
         </is>
       </c>
-      <c r="B38" s="26" t="n"/>
-      <c r="C38" s="26" t="n"/>
-      <c r="D38" s="26" t="n"/>
-      <c r="E38" s="26" t="n"/>
-      <c r="F38" s="26" t="n"/>
-      <c r="G38" s="26" t="n"/>
+      <c r="B38" s="29" t="n"/>
+      <c r="C38" s="29" t="n"/>
+      <c r="D38" s="29" t="n"/>
+      <c r="E38" s="29" t="n"/>
+      <c r="F38" s="29" t="n"/>
+      <c r="G38" s="30" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="26" t="inlineStr">
@@ -3216,12 +3246,12 @@
           <t>▶ pet_care_records</t>
         </is>
       </c>
-      <c r="B51" s="26" t="n"/>
-      <c r="C51" s="26" t="n"/>
-      <c r="D51" s="26" t="n"/>
-      <c r="E51" s="26" t="n"/>
-      <c r="F51" s="26" t="n"/>
-      <c r="G51" s="26" t="n"/>
+      <c r="B51" s="29" t="n"/>
+      <c r="C51" s="29" t="n"/>
+      <c r="D51" s="29" t="n"/>
+      <c r="E51" s="29" t="n"/>
+      <c r="F51" s="29" t="n"/>
+      <c r="G51" s="30" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="26" t="inlineStr">
@@ -3489,12 +3519,12 @@
           <t>▶ symptom_checks</t>
         </is>
       </c>
-      <c r="B60" s="26" t="n"/>
-      <c r="C60" s="26" t="n"/>
-      <c r="D60" s="26" t="n"/>
-      <c r="E60" s="26" t="n"/>
-      <c r="F60" s="26" t="n"/>
-      <c r="G60" s="26" t="n"/>
+      <c r="B60" s="29" t="n"/>
+      <c r="C60" s="29" t="n"/>
+      <c r="D60" s="29" t="n"/>
+      <c r="E60" s="29" t="n"/>
+      <c r="F60" s="29" t="n"/>
+      <c r="G60" s="30" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="26" t="inlineStr">
@@ -3733,12 +3763,12 @@
           <t>▶ plans</t>
         </is>
       </c>
-      <c r="B68" s="26" t="n"/>
-      <c r="C68" s="26" t="n"/>
-      <c r="D68" s="26" t="n"/>
-      <c r="E68" s="26" t="n"/>
-      <c r="F68" s="26" t="n"/>
-      <c r="G68" s="26" t="n"/>
+      <c r="B68" s="29" t="n"/>
+      <c r="C68" s="29" t="n"/>
+      <c r="D68" s="29" t="n"/>
+      <c r="E68" s="29" t="n"/>
+      <c r="F68" s="29" t="n"/>
+      <c r="G68" s="30" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="26" t="inlineStr">
@@ -4010,12 +4040,12 @@
           <t>▶ plan_features</t>
         </is>
       </c>
-      <c r="B77" s="26" t="n"/>
-      <c r="C77" s="26" t="n"/>
-      <c r="D77" s="26" t="n"/>
-      <c r="E77" s="26" t="n"/>
-      <c r="F77" s="26" t="n"/>
-      <c r="G77" s="26" t="n"/>
+      <c r="B77" s="29" t="n"/>
+      <c r="C77" s="29" t="n"/>
+      <c r="D77" s="29" t="n"/>
+      <c r="E77" s="29" t="n"/>
+      <c r="F77" s="29" t="n"/>
+      <c r="G77" s="30" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="26" t="inlineStr">
@@ -4089,12 +4119,12 @@
           <t>▶ subscriptions</t>
         </is>
       </c>
-      <c r="B80" s="26" t="n"/>
-      <c r="C80" s="26" t="n"/>
-      <c r="D80" s="26" t="n"/>
-      <c r="E80" s="26" t="n"/>
-      <c r="F80" s="26" t="n"/>
-      <c r="G80" s="26" t="n"/>
+      <c r="B80" s="29" t="n"/>
+      <c r="C80" s="29" t="n"/>
+      <c r="D80" s="29" t="n"/>
+      <c r="E80" s="29" t="n"/>
+      <c r="F80" s="29" t="n"/>
+      <c r="G80" s="30" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="26" t="inlineStr">
@@ -4465,12 +4495,12 @@
           <t>▶ invoices</t>
         </is>
       </c>
-      <c r="B92" s="26" t="n"/>
-      <c r="C92" s="26" t="n"/>
-      <c r="D92" s="26" t="n"/>
-      <c r="E92" s="26" t="n"/>
-      <c r="F92" s="26" t="n"/>
-      <c r="G92" s="26" t="n"/>
+      <c r="B92" s="29" t="n"/>
+      <c r="C92" s="29" t="n"/>
+      <c r="D92" s="29" t="n"/>
+      <c r="E92" s="29" t="n"/>
+      <c r="F92" s="29" t="n"/>
+      <c r="G92" s="30" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="26" t="inlineStr">
@@ -4771,12 +4801,12 @@
           <t>▶ payments</t>
         </is>
       </c>
-      <c r="B102" s="26" t="n"/>
-      <c r="C102" s="26" t="n"/>
-      <c r="D102" s="26" t="n"/>
-      <c r="E102" s="26" t="n"/>
-      <c r="F102" s="26" t="n"/>
-      <c r="G102" s="26" t="n"/>
+      <c r="B102" s="29" t="n"/>
+      <c r="C102" s="29" t="n"/>
+      <c r="D102" s="29" t="n"/>
+      <c r="E102" s="29" t="n"/>
+      <c r="F102" s="29" t="n"/>
+      <c r="G102" s="30" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="26" t="inlineStr">
@@ -4982,12 +5012,12 @@
           <t>▶ appointment_slots</t>
         </is>
       </c>
-      <c r="B109" s="26" t="n"/>
-      <c r="C109" s="26" t="n"/>
-      <c r="D109" s="26" t="n"/>
-      <c r="E109" s="26" t="n"/>
-      <c r="F109" s="26" t="n"/>
-      <c r="G109" s="26" t="n"/>
+      <c r="B109" s="29" t="n"/>
+      <c r="C109" s="29" t="n"/>
+      <c r="D109" s="29" t="n"/>
+      <c r="E109" s="29" t="n"/>
+      <c r="F109" s="29" t="n"/>
+      <c r="G109" s="30" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="26" t="inlineStr">
@@ -5251,12 +5281,12 @@
           <t>▶ appointments</t>
         </is>
       </c>
-      <c r="B118" s="26" t="n"/>
-      <c r="C118" s="26" t="n"/>
-      <c r="D118" s="26" t="n"/>
-      <c r="E118" s="26" t="n"/>
-      <c r="F118" s="26" t="n"/>
-      <c r="G118" s="26" t="n"/>
+      <c r="B118" s="29" t="n"/>
+      <c r="C118" s="29" t="n"/>
+      <c r="D118" s="29" t="n"/>
+      <c r="E118" s="29" t="n"/>
+      <c r="F118" s="29" t="n"/>
+      <c r="G118" s="30" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="26" t="inlineStr">
@@ -5660,12 +5690,12 @@
           <t>▶ medical_histories</t>
         </is>
       </c>
-      <c r="B131" s="26" t="n"/>
-      <c r="C131" s="26" t="n"/>
-      <c r="D131" s="26" t="n"/>
-      <c r="E131" s="26" t="n"/>
-      <c r="F131" s="26" t="n"/>
-      <c r="G131" s="26" t="n"/>
+      <c r="B131" s="29" t="n"/>
+      <c r="C131" s="29" t="n"/>
+      <c r="D131" s="29" t="n"/>
+      <c r="E131" s="29" t="n"/>
+      <c r="F131" s="29" t="n"/>
+      <c r="G131" s="30" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="26" t="inlineStr">
@@ -6073,12 +6103,12 @@
           <t>▶ medical_attachments</t>
         </is>
       </c>
-      <c r="B144" s="26" t="n"/>
-      <c r="C144" s="26" t="n"/>
-      <c r="D144" s="26" t="n"/>
-      <c r="E144" s="26" t="n"/>
-      <c r="F144" s="26" t="n"/>
-      <c r="G144" s="26" t="n"/>
+      <c r="B144" s="29" t="n"/>
+      <c r="C144" s="29" t="n"/>
+      <c r="D144" s="29" t="n"/>
+      <c r="E144" s="29" t="n"/>
+      <c r="F144" s="29" t="n"/>
+      <c r="G144" s="30" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="26" t="inlineStr">
@@ -6251,12 +6281,12 @@
           <t>▶ consult_chat_messages</t>
         </is>
       </c>
-      <c r="B150" s="26" t="n"/>
-      <c r="C150" s="26" t="n"/>
-      <c r="D150" s="26" t="n"/>
-      <c r="E150" s="26" t="n"/>
-      <c r="F150" s="26" t="n"/>
-      <c r="G150" s="26" t="n"/>
+      <c r="B150" s="29" t="n"/>
+      <c r="C150" s="29" t="n"/>
+      <c r="D150" s="29" t="n"/>
+      <c r="E150" s="29" t="n"/>
+      <c r="F150" s="29" t="n"/>
+      <c r="G150" s="30" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="26" t="inlineStr">
@@ -6454,12 +6484,12 @@
           <t>▶ notifications</t>
         </is>
       </c>
-      <c r="B157" s="26" t="n"/>
-      <c r="C157" s="26" t="n"/>
-      <c r="D157" s="26" t="n"/>
-      <c r="E157" s="26" t="n"/>
-      <c r="F157" s="26" t="n"/>
-      <c r="G157" s="26" t="n"/>
+      <c r="B157" s="29" t="n"/>
+      <c r="C157" s="29" t="n"/>
+      <c r="D157" s="29" t="n"/>
+      <c r="E157" s="29" t="n"/>
+      <c r="F157" s="29" t="n"/>
+      <c r="G157" s="30" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="26" t="inlineStr">
@@ -6628,12 +6658,12 @@
           <t>▶ notification_recipients</t>
         </is>
       </c>
-      <c r="B163" s="26" t="n"/>
-      <c r="C163" s="26" t="n"/>
-      <c r="D163" s="26" t="n"/>
-      <c r="E163" s="26" t="n"/>
-      <c r="F163" s="26" t="n"/>
-      <c r="G163" s="26" t="n"/>
+      <c r="B163" s="29" t="n"/>
+      <c r="C163" s="29" t="n"/>
+      <c r="D163" s="29" t="n"/>
+      <c r="E163" s="29" t="n"/>
+      <c r="F163" s="29" t="n"/>
+      <c r="G163" s="30" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="26" t="inlineStr">
@@ -6773,12 +6803,12 @@
           <t>▶ email_templates</t>
         </is>
       </c>
-      <c r="B168" s="26" t="n"/>
-      <c r="C168" s="26" t="n"/>
-      <c r="D168" s="26" t="n"/>
-      <c r="E168" s="26" t="n"/>
-      <c r="F168" s="26" t="n"/>
-      <c r="G168" s="26" t="n"/>
+      <c r="B168" s="29" t="n"/>
+      <c r="C168" s="29" t="n"/>
+      <c r="D168" s="29" t="n"/>
+      <c r="E168" s="29" t="n"/>
+      <c r="F168" s="29" t="n"/>
+      <c r="G168" s="30" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="26" t="inlineStr">
@@ -6980,12 +7010,12 @@
           <t>▶ email_messages</t>
         </is>
       </c>
-      <c r="B175" s="26" t="n"/>
-      <c r="C175" s="26" t="n"/>
-      <c r="D175" s="26" t="n"/>
-      <c r="E175" s="26" t="n"/>
-      <c r="F175" s="26" t="n"/>
-      <c r="G175" s="26" t="n"/>
+      <c r="B175" s="29" t="n"/>
+      <c r="C175" s="29" t="n"/>
+      <c r="D175" s="29" t="n"/>
+      <c r="E175" s="29" t="n"/>
+      <c r="F175" s="29" t="n"/>
+      <c r="G175" s="30" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="26" t="inlineStr">
@@ -7253,12 +7283,12 @@
           <t>▶ pet_calendar_marks</t>
         </is>
       </c>
-      <c r="B184" s="26" t="n"/>
-      <c r="C184" s="26" t="n"/>
-      <c r="D184" s="26" t="n"/>
-      <c r="E184" s="26" t="n"/>
-      <c r="F184" s="26" t="n"/>
-      <c r="G184" s="26" t="n"/>
+      <c r="B184" s="29" t="n"/>
+      <c r="C184" s="29" t="n"/>
+      <c r="D184" s="29" t="n"/>
+      <c r="E184" s="29" t="n"/>
+      <c r="F184" s="29" t="n"/>
+      <c r="G184" s="30" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="26" t="inlineStr">
@@ -7530,12 +7560,12 @@
           <t>▶ dismissed_reminders</t>
         </is>
       </c>
-      <c r="B193" s="26" t="n"/>
-      <c r="C193" s="26" t="n"/>
-      <c r="D193" s="26" t="n"/>
-      <c r="E193" s="26" t="n"/>
-      <c r="F193" s="26" t="n"/>
-      <c r="G193" s="26" t="n"/>
+      <c r="B193" s="29" t="n"/>
+      <c r="C193" s="29" t="n"/>
+      <c r="D193" s="29" t="n"/>
+      <c r="E193" s="29" t="n"/>
+      <c r="F193" s="29" t="n"/>
+      <c r="G193" s="30" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="26" t="inlineStr">
@@ -7679,12 +7709,12 @@
           <t>▶ announcements</t>
         </is>
       </c>
-      <c r="B198" s="26" t="n"/>
-      <c r="C198" s="26" t="n"/>
-      <c r="D198" s="26" t="n"/>
-      <c r="E198" s="26" t="n"/>
-      <c r="F198" s="26" t="n"/>
-      <c r="G198" s="26" t="n"/>
+      <c r="B198" s="29" t="n"/>
+      <c r="C198" s="29" t="n"/>
+      <c r="D198" s="29" t="n"/>
+      <c r="E198" s="29" t="n"/>
+      <c r="F198" s="29" t="n"/>
+      <c r="G198" s="30" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="26" t="inlineStr">
@@ -7919,12 +7949,12 @@
           <t>▶ password_reset_tokens</t>
         </is>
       </c>
-      <c r="B206" s="26" t="n"/>
-      <c r="C206" s="26" t="n"/>
-      <c r="D206" s="26" t="n"/>
-      <c r="E206" s="26" t="n"/>
-      <c r="F206" s="26" t="n"/>
-      <c r="G206" s="26" t="n"/>
+      <c r="B206" s="29" t="n"/>
+      <c r="C206" s="29" t="n"/>
+      <c r="D206" s="29" t="n"/>
+      <c r="E206" s="29" t="n"/>
+      <c r="F206" s="29" t="n"/>
+      <c r="G206" s="30" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="26" t="inlineStr">
@@ -8216,10 +8246,10 @@
           <t>── Auth（認証） ──</t>
         </is>
       </c>
-      <c r="B4" s="26" t="n"/>
-      <c r="C4" s="26" t="n"/>
-      <c r="D4" s="26" t="n"/>
-      <c r="E4" s="26" t="n"/>
+      <c r="B4" s="29" t="n"/>
+      <c r="C4" s="29" t="n"/>
+      <c r="D4" s="29" t="n"/>
+      <c r="E4" s="30" t="n"/>
     </row>
     <row r="5" ht="15" customHeight="1" s="12">
       <c r="A5" s="26" t="inlineStr">
@@ -8335,10 +8365,10 @@
           <t>── ペット・健康管理 ──</t>
         </is>
       </c>
-      <c r="B9" s="26" t="n"/>
-      <c r="C9" s="26" t="n"/>
-      <c r="D9" s="26" t="n"/>
-      <c r="E9" s="26" t="n"/>
+      <c r="B9" s="29" t="n"/>
+      <c r="C9" s="29" t="n"/>
+      <c r="D9" s="29" t="n"/>
+      <c r="E9" s="30" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1" s="12">
       <c r="A10" s="26" t="inlineStr">
@@ -8481,10 +8511,10 @@
           <t>── プラン・課金 ──</t>
         </is>
       </c>
-      <c r="B15" s="26" t="n"/>
-      <c r="C15" s="26" t="n"/>
-      <c r="D15" s="26" t="n"/>
-      <c r="E15" s="26" t="n"/>
+      <c r="B15" s="29" t="n"/>
+      <c r="C15" s="29" t="n"/>
+      <c r="D15" s="29" t="n"/>
+      <c r="E15" s="30" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="26" t="inlineStr">
@@ -8681,10 +8711,10 @@
           <t>── 予約・診療記録 ──</t>
         </is>
       </c>
-      <c r="B23" s="26" t="n"/>
-      <c r="C23" s="26" t="n"/>
-      <c r="D23" s="26" t="n"/>
-      <c r="E23" s="26" t="n"/>
+      <c r="B23" s="29" t="n"/>
+      <c r="C23" s="29" t="n"/>
+      <c r="D23" s="29" t="n"/>
+      <c r="E23" s="30" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="26" t="inlineStr">
@@ -8908,10 +8938,10 @@
           <t>── メッセージング・通知 ──</t>
         </is>
       </c>
-      <c r="B32" s="26" t="n"/>
-      <c r="C32" s="26" t="n"/>
-      <c r="D32" s="26" t="n"/>
-      <c r="E32" s="26" t="n"/>
+      <c r="B32" s="29" t="n"/>
+      <c r="C32" s="29" t="n"/>
+      <c r="D32" s="29" t="n"/>
+      <c r="E32" s="30" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="26" t="inlineStr">
@@ -9108,10 +9138,10 @@
           <t>── UX補助 ──</t>
         </is>
       </c>
-      <c r="B40" s="26" t="n"/>
-      <c r="C40" s="26" t="n"/>
-      <c r="D40" s="26" t="n"/>
-      <c r="E40" s="26" t="n"/>
+      <c r="B40" s="29" t="n"/>
+      <c r="C40" s="29" t="n"/>
+      <c r="D40" s="29" t="n"/>
+      <c r="E40" s="30" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="26" t="inlineStr">
@@ -9574,51 +9604,51 @@
     <row r="22" ht="15" customHeight="1" s="12">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>admin@petlifeplus.local</t>
+          <t>super@petlife.local</t>
         </is>
       </c>
       <c r="B22" s="26" t="inlineStr">
         <is>
-          <t>admin123</t>
+          <t>super123</t>
         </is>
       </c>
       <c r="C22" s="26" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>SUPER</t>
         </is>
       </c>
       <c r="D22" s="26" t="inlineStr">
         <is>
-          <t>管理者</t>
+          <t>開発者（全権限）</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="12">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>owner1@petlifeplus.local</t>
+          <t>admin@petlife.local</t>
         </is>
       </c>
       <c r="B23" s="26" t="inlineStr">
         <is>
-          <t>user123</t>
+          <t>admin123</t>
         </is>
       </c>
       <c r="C23" s="26" t="inlineStr">
         <is>
-          <t>USER</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="D23" s="26" t="inlineStr">
         <is>
-          <t>一般ユーザー（プレミアム）</t>
+          <t>管理者</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="12">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t>vet1@petlifeplus.local</t>
+          <t>vet1@petlife.local</t>
         </is>
       </c>
       <c r="B24" s="26" t="inlineStr">
@@ -9640,7 +9670,7 @@
     <row r="25" ht="15" customHeight="1" s="12">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>staff1@petlifeplus.local</t>
+          <t>staff1@petlife.local</t>
         </is>
       </c>
       <c r="B25" s="26" t="inlineStr">
@@ -9662,7 +9692,7 @@
     <row r="26" ht="15" customHeight="1" s="12">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>owner2@petlifeplus.local</t>
+          <t>owner1@petlife.local</t>
         </is>
       </c>
       <c r="B26" s="26" t="inlineStr">
@@ -9677,19 +9707,19 @@
       </c>
       <c r="D26" s="26" t="inlineStr">
         <is>
-          <t>一般ユーザー（スタンダード）</t>
+          <t>一般ユーザー（ライト）</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="12">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>owner.light@petlifeplus.local</t>
+          <t>owner2@petlife.local</t>
         </is>
       </c>
       <c r="B27" s="26" t="inlineStr">
         <is>
-          <t>light123</t>
+          <t>user123</t>
         </is>
       </c>
       <c r="C27" s="26" t="inlineStr">
@@ -9699,19 +9729,19 @@
       </c>
       <c r="D27" s="26" t="inlineStr">
         <is>
-          <t>ライトプランユーザー</t>
+          <t>一般ユーザー（スタンダード）</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="12">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>owner.standard@petlifeplus.local</t>
+          <t>owner3@petlife.local</t>
         </is>
       </c>
       <c r="B28" s="26" t="inlineStr">
         <is>
-          <t>standard123</t>
+          <t>user123</t>
         </is>
       </c>
       <c r="C28" s="26" t="inlineStr">
@@ -9721,31 +9751,15 @@
       </c>
       <c r="D28" s="26" t="inlineStr">
         <is>
-          <t>スタンダードプランユーザー</t>
+          <t>一般ユーザー（プレミアム）</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="12">
-      <c r="A29" s="26" t="inlineStr">
-        <is>
-          <t>owner.premium@petlifeplus.local</t>
-        </is>
-      </c>
-      <c r="B29" s="26" t="inlineStr">
-        <is>
-          <t>premium123</t>
-        </is>
-      </c>
-      <c r="C29" s="26" t="inlineStr">
-        <is>
-          <t>USER</t>
-        </is>
-      </c>
-      <c r="D29" s="26" t="inlineStr">
-        <is>
-          <t>プレミアムプランユーザー</t>
-        </is>
-      </c>
+      <c r="A29" s="26" t="inlineStr"/>
+      <c r="B29" s="26" t="inlineStr"/>
+      <c r="C29" s="26" t="inlineStr"/>
+      <c r="D29" s="26" t="inlineStr"/>
     </row>
     <row r="30" ht="15" customHeight="1" s="12"/>
     <row r="31" ht="15" customHeight="1" s="12"/>
@@ -9787,7 +9801,7 @@
       </c>
       <c r="C34" s="26" t="inlineStr">
         <is>
-          <t>各ユーザーの飼いペット（犬・猫）</t>
+          <t>ポチ/タロウ/レオン/ピーコ/カレン/ボス（すべて犬）</t>
         </is>
       </c>
       <c r="D34" s="26" t="inlineStr"/>
@@ -9805,7 +9819,7 @@
       </c>
       <c r="C35" s="26" t="inlineStr">
         <is>
-          <t>ペット1〜3の健康記録</t>
+          <t>ペット1～3の健康記録</t>
         </is>
       </c>
       <c r="D35" s="26" t="inlineStr"/>
@@ -9823,7 +9837,7 @@
       </c>
       <c r="C36" s="26" t="inlineStr">
         <is>
-          <t>ペット1〜3のケア記録</t>
+          <t>ポチのケア記録（3件）</t>
         </is>
       </c>
       <c r="D36" s="26" t="inlineStr"/>
@@ -9841,7 +9855,7 @@
       </c>
       <c r="C37" s="26" t="inlineStr">
         <is>
-          <t>各プランへの契約</t>
+          <t>owner1→ポチ(STANDARD)、owner2→レオン(STANDARD)、owner1→ピーコ(LIGHT)、owner2→カレン(STANDARD)、owner3→ボス(PREMIUM)</t>
         </is>
       </c>
       <c r="D37" s="26" t="inlineStr"/>

</xml_diff>